<commit_message>
Updated savedata function to save in correct file location
</commit_message>
<xml_diff>
--- a/MATLAB Files/Results/Run Log.xlsx
+++ b/MATLAB Files/Results/Run Log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="17" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="27" uniqueCount="9">
   <si>
     <t>RunID</t>
   </si>
@@ -86,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="true"/>
@@ -95,7 +95,7 @@
     <col min="4" max="4" width="14.21875" customWidth="true"/>
     <col min="5" max="5" width="16.109375" customWidth="true"/>
     <col min="6" max="6" width="8" customWidth="true"/>
-    <col min="7" max="7" width="5.6640625" customWidth="true"/>
+    <col min="7" max="7" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -167,6 +167,29 @@
         <v>11.401754250991379</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46211.739891338053</v>
+      </c>
+      <c r="C4" s="0">
+        <v>0.45000000000000001</v>
+      </c>
+      <c r="D4" s="0">
+        <v>1.3</v>
+      </c>
+      <c r="E4" s="0">
+        <v>0.01</v>
+      </c>
+      <c r="F4" s="0">
+        <v>100</v>
+      </c>
+      <c r="G4" s="0">
+        <v>11.401754250991379</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added results table function for global results collection and updated homing loop code
</commit_message>
<xml_diff>
--- a/MATLAB Files/Results/Run Log.xlsx
+++ b/MATLAB Files/Results/Run Log.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="low_pass_filter_white_noise" sheetId="1" r:id="rId2"/>
+    <sheet name="homing_loop_covariance_analysis" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="27" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="92" uniqueCount="18">
   <si>
     <t>RunID</t>
   </si>
@@ -41,6 +42,33 @@
   </si>
   <si>
     <t>1487113365</t>
+  </si>
+  <si>
+    <t>1494086941</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>nav_ratio</t>
+  </si>
+  <si>
+    <t>time_constant</t>
+  </si>
+  <si>
+    <t>closing_vel_mps</t>
+  </si>
+  <si>
+    <t>target_accel_mps2</t>
+  </si>
+  <si>
+    <t>t_initial_s</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>1016206606</t>
   </si>
 </sst>
 </file>
@@ -192,4 +220,217 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="true"/>
+    <col min="2" max="2" width="15.5546875" customWidth="true"/>
+    <col min="3" max="3" width="4.5546875" customWidth="true"/>
+    <col min="4" max="4" width="8.77734375" customWidth="true"/>
+    <col min="5" max="5" width="12.77734375" customWidth="true"/>
+    <col min="6" max="6" width="8" customWidth="true"/>
+    <col min="7" max="7" width="14.21875" customWidth="true"/>
+    <col min="8" max="8" width="16.44140625" customWidth="true"/>
+    <col min="9" max="9" width="8.88671875" customWidth="true"/>
+    <col min="10" max="10" width="6.5546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46212.619980270713</v>
+      </c>
+      <c r="C2" s="0">
+        <v>9.8100000000000005</v>
+      </c>
+      <c r="D2" s="0">
+        <v>5</v>
+      </c>
+      <c r="E2" s="0">
+        <v>1</v>
+      </c>
+      <c r="F2" s="0">
+        <v>10</v>
+      </c>
+      <c r="G2" s="0">
+        <v>4000</v>
+      </c>
+      <c r="H2" s="0">
+        <v>29.43</v>
+      </c>
+      <c r="I2" s="0">
+        <v>1.0000000000000001e-05</v>
+      </c>
+      <c r="J2" s="0">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46212.620939847133</v>
+      </c>
+      <c r="C3" s="0">
+        <v>9.8100000000000005</v>
+      </c>
+      <c r="D3" s="0">
+        <v>3</v>
+      </c>
+      <c r="E3" s="0">
+        <v>1</v>
+      </c>
+      <c r="F3" s="0">
+        <v>10</v>
+      </c>
+      <c r="G3" s="0">
+        <v>1219</v>
+      </c>
+      <c r="H3" s="0">
+        <v>29.43</v>
+      </c>
+      <c r="I3" s="0">
+        <v>1.0000000000000001e-05</v>
+      </c>
+      <c r="J3" s="0">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46212.682414040523</v>
+      </c>
+      <c r="C4" s="0">
+        <v>9.8100000000000005</v>
+      </c>
+      <c r="D4" s="0">
+        <v>3</v>
+      </c>
+      <c r="E4" s="0">
+        <v>1</v>
+      </c>
+      <c r="F4" s="0">
+        <v>10</v>
+      </c>
+      <c r="G4" s="0">
+        <v>1219</v>
+      </c>
+      <c r="H4" s="0">
+        <v>29.43</v>
+      </c>
+      <c r="I4" s="0">
+        <v>1.0000000000000001e-05</v>
+      </c>
+      <c r="J4" s="0">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46212.690953813864</v>
+      </c>
+      <c r="C5" s="0">
+        <v>9.8100000000000005</v>
+      </c>
+      <c r="D5" s="0">
+        <v>3</v>
+      </c>
+      <c r="E5" s="0">
+        <v>1</v>
+      </c>
+      <c r="F5" s="0">
+        <v>10</v>
+      </c>
+      <c r="G5" s="0">
+        <v>1219</v>
+      </c>
+      <c r="H5" s="0">
+        <v>29.43</v>
+      </c>
+      <c r="I5" s="0">
+        <v>1.0000000000000001e-05</v>
+      </c>
+      <c r="J5" s="0">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46212.691423446864</v>
+      </c>
+      <c r="C6" s="0">
+        <v>9.8100000000000005</v>
+      </c>
+      <c r="D6" s="0">
+        <v>3</v>
+      </c>
+      <c r="E6" s="0">
+        <v>1</v>
+      </c>
+      <c r="F6" s="0">
+        <v>10</v>
+      </c>
+      <c r="G6" s="0">
+        <v>1219</v>
+      </c>
+      <c r="H6" s="0">
+        <v>29.43</v>
+      </c>
+      <c r="I6" s="0">
+        <v>1.0000000000000001e-05</v>
+      </c>
+      <c r="J6" s="0">
+        <v>0.0001</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added acceleration and miss distance adjoint code
</commit_message>
<xml_diff>
--- a/MATLAB Files/Results/Run Log.xlsx
+++ b/MATLAB Files/Results/Run Log.xlsx
@@ -1,21 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fileVersion appName="libxl" rupBuild="4.6.0"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="libxl" lastEdited="7" lowestEdited="7" rupBuild="4.6.0"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benme\Github_Code\Tactical and Strategic Missile Guidance\MATLAB Files\Results\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612E93A4-5A4B-48C8-B29F-7E15B291C14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="low_pass_filter_white_noise" sheetId="1" r:id="rId2"/>
-    <sheet name="homing_loop_covariance_analysis" sheetId="2" r:id="rId4"/>
+    <sheet name="low_pass_filter_white_noise" sheetId="1" r:id="rId1"/>
+    <sheet name="homing_loop_covariance_analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="accel_miss_dist_adjoint" sheetId="3" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="92" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="76" uniqueCount="24">
   <si>
     <t>RunID</t>
   </si>
@@ -44,9 +51,6 @@
     <t>1487113365</t>
   </si>
   <si>
-    <t>1494086941</t>
-  </si>
-  <si>
     <t>G</t>
   </si>
   <si>
@@ -69,6 +73,27 @@
   </si>
   <si>
     <t>1016206606</t>
+  </si>
+  <si>
+    <t>1878749455</t>
+  </si>
+  <si>
+    <t>missile_accel_mps2</t>
+  </si>
+  <si>
+    <t>640197084</t>
+  </si>
+  <si>
+    <t>t_int</t>
+  </si>
+  <si>
+    <t>miss</t>
+  </si>
+  <si>
+    <t>32120221</t>
+  </si>
+  <si>
+    <t>1383544862</t>
   </si>
 </sst>
 </file>
@@ -97,25 +122,356 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="true">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="false"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="true">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="false"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="true">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="false"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="true"/>
     <col min="2" max="2" width="15.5546875" customWidth="true"/>
@@ -126,7 +482,7 @@
     <col min="7" max="7" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
@@ -149,7 +505,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
@@ -172,7 +528,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="0" t="s">
         <v>8</v>
       </c>
@@ -195,7 +551,7 @@
         <v>11.401754250991379</v>
       </c>
     </row>
-    <row r="4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="0" t="s">
         <v>8</v>
       </c>
@@ -218,25 +574,271 @@
         <v>11.401754250991379</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46212.822921438194</v>
+      </c>
+      <c r="C5" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="D5" s="0">
+        <v>1</v>
+      </c>
+      <c r="E5" s="0">
+        <v>0.01</v>
+      </c>
+      <c r="F5" s="0">
+        <v>100</v>
+      </c>
+      <c r="G5" s="0">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.88671875" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="3" max="3" width="2.21875" customWidth="1"/>
+    <col min="4" max="4" width="8.77734375" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="14.21875" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
+    <col min="10" max="10" width="2" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46212.743425844368</v>
+      </c>
+      <c r="C2">
+        <v>9.81</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>1219</v>
+      </c>
+      <c r="H2">
+        <v>29.43</v>
+      </c>
+      <c r="I2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J2">
+        <v>1E-4</v>
+      </c>
+      <c r="K2">
+        <v>392.40000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46212.620939847133</v>
+      </c>
+      <c r="C3">
+        <v>9.81</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>1219</v>
+      </c>
+      <c r="H3">
+        <v>29.43</v>
+      </c>
+      <c r="I3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J3">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46212.682414040522</v>
+      </c>
+      <c r="C4">
+        <v>9.81</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>1219</v>
+      </c>
+      <c r="H4">
+        <v>29.43</v>
+      </c>
+      <c r="I4">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J4">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46212.690953813864</v>
+      </c>
+      <c r="C5">
+        <v>9.81</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>1219</v>
+      </c>
+      <c r="H5">
+        <v>29.43</v>
+      </c>
+      <c r="I5">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J5">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46212.691423446864</v>
+      </c>
+      <c r="C6">
+        <v>9.81</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>1219</v>
+      </c>
+      <c r="H6">
+        <v>29.43</v>
+      </c>
+      <c r="I6">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J6">
+        <v>1E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="true"/>
+    <col min="1" max="1" width="10" customWidth="true"/>
     <col min="2" max="2" width="15.5546875" customWidth="true"/>
     <col min="3" max="3" width="4.5546875" customWidth="true"/>
     <col min="4" max="4" width="8.77734375" customWidth="true"/>
     <col min="5" max="5" width="12.77734375" customWidth="true"/>
     <col min="6" max="6" width="8" customWidth="true"/>
-    <col min="7" max="7" width="14.21875" customWidth="true"/>
+    <col min="7" max="7" width="4.77734375" customWidth="true"/>
     <col min="8" max="8" width="16.44140625" customWidth="true"/>
     <col min="9" max="9" width="8.88671875" customWidth="true"/>
     <col min="10" max="10" width="6.5546875" customWidth="true"/>
+    <col min="11" max="11" width="4.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -247,42 +849,45 @@
         <v>2</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="0" t="s">
         <v>11</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>12</v>
       </c>
       <c r="F1" s="0" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="I1" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="J1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="0" t="s">
-        <v>16</v>
+      <c r="K1" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1">
-        <v>46212.619980270713</v>
+        <v>46212.802283827288</v>
       </c>
       <c r="C2" s="0">
         <v>9.8100000000000005</v>
       </c>
       <c r="D2" s="0">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E2" s="0">
         <v>1</v>
@@ -291,7 +896,7 @@
         <v>10</v>
       </c>
       <c r="G2" s="0">
-        <v>4000</v>
+        <v>1</v>
       </c>
       <c r="H2" s="0">
         <v>29.43</v>
@@ -302,13 +907,16 @@
       <c r="J2" s="0">
         <v>0.0001</v>
       </c>
+      <c r="K2" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1">
-        <v>46212.620939847133</v>
+        <v>46212.802345490047</v>
       </c>
       <c r="C3" s="0">
         <v>9.8100000000000005</v>
@@ -323,7 +931,7 @@
         <v>10</v>
       </c>
       <c r="G3" s="0">
-        <v>1219</v>
+        <v>2</v>
       </c>
       <c r="H3" s="0">
         <v>29.43</v>
@@ -334,13 +942,16 @@
       <c r="J3" s="0">
         <v>0.0001</v>
       </c>
+      <c r="K3" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B4" s="1">
-        <v>46212.682414040523</v>
+        <v>46212.802401839173</v>
       </c>
       <c r="C4" s="0">
         <v>9.8100000000000005</v>
@@ -355,7 +966,7 @@
         <v>10</v>
       </c>
       <c r="G4" s="0">
-        <v>1219</v>
+        <v>0.5</v>
       </c>
       <c r="H4" s="0">
         <v>29.43</v>
@@ -366,69 +977,8 @@
       <c r="J4" s="0">
         <v>0.0001</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="1">
-        <v>46212.690953813864</v>
-      </c>
-      <c r="C5" s="0">
-        <v>9.8100000000000005</v>
-      </c>
-      <c r="D5" s="0">
-        <v>3</v>
-      </c>
-      <c r="E5" s="0">
-        <v>1</v>
-      </c>
-      <c r="F5" s="0">
-        <v>10</v>
-      </c>
-      <c r="G5" s="0">
-        <v>1219</v>
-      </c>
-      <c r="H5" s="0">
-        <v>29.43</v>
-      </c>
-      <c r="I5" s="0">
-        <v>1.0000000000000001e-05</v>
-      </c>
-      <c r="J5" s="0">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="1">
-        <v>46212.691423446864</v>
-      </c>
-      <c r="C6" s="0">
-        <v>9.8100000000000005</v>
-      </c>
-      <c r="D6" s="0">
-        <v>3</v>
-      </c>
-      <c r="E6" s="0">
-        <v>1</v>
-      </c>
-      <c r="F6" s="0">
-        <v>10</v>
-      </c>
-      <c r="G6" s="0">
-        <v>1219</v>
-      </c>
-      <c r="H6" s="0">
-        <v>29.43</v>
-      </c>
-      <c r="I6" s="0">
-        <v>1.0000000000000001e-05</v>
-      </c>
-      <c r="J6" s="0">
-        <v>0.0001</v>
+      <c r="K4" s="0">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rewrote from first principles non-linear proportional navigation homing loop
</commit_message>
<xml_diff>
--- a/MATLAB Files/Results/Run Log.xlsx
+++ b/MATLAB Files/Results/Run Log.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benme\Github_Code\Tactical and Strategic Missile Guidance\MATLAB Files\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612E93A4-5A4B-48C8-B29F-7E15B291C14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15889988-C117-49E9-8CFD-04E5A67F176F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="low_pass_filter_white_noise" sheetId="1" r:id="rId1"/>
     <sheet name="homing_loop_covariance_analysis" sheetId="2" r:id="rId2"/>
-    <sheet name="accel_miss_dist_adjoint" sheetId="3" r:id="rId6"/>
+    <sheet name="accel_miss_dist_adjoint" sheetId="3" r:id="rId3"/>
+    <sheet name="proportional_nav_homing_loop" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="76" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="223" uniqueCount="46">
   <si>
     <t>RunID</t>
   </si>
@@ -94,6 +95,72 @@
   </si>
   <si>
     <t>1383544862</t>
+  </si>
+  <si>
+    <t>608216979</t>
+  </si>
+  <si>
+    <t>161090779</t>
+  </si>
+  <si>
+    <t>2058745317</t>
+  </si>
+  <si>
+    <t>seed</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>missile_vel</t>
+  </si>
+  <si>
+    <t>target_vel</t>
+  </si>
+  <si>
+    <t>heading_err</t>
+  </si>
+  <si>
+    <t>missile_pos_1</t>
+  </si>
+  <si>
+    <t>missile_pos_2</t>
+  </si>
+  <si>
+    <t>target_pos_1</t>
+  </si>
+  <si>
+    <t>target_pos_2</t>
+  </si>
+  <si>
+    <t>beta</t>
+  </si>
+  <si>
+    <t>missile_max_accel</t>
+  </si>
+  <si>
+    <t>731042643</t>
+  </si>
+  <si>
+    <t>231072461</t>
+  </si>
+  <si>
+    <t>1010079013</t>
+  </si>
+  <si>
+    <t>784456645</t>
+  </si>
+  <si>
+    <t>1878011713</t>
+  </si>
+  <si>
+    <t>1721021967</t>
+  </si>
+  <si>
+    <t>1085451352</t>
+  </si>
+  <si>
+    <t>693683582</t>
   </si>
 </sst>
 </file>
@@ -470,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="true"/>
@@ -483,117 +550,163 @@
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="0" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" t="s">
         <v>7</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
-      <c r="A2" s="0" t="s">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1">
         <v>46211.737071405325</v>
       </c>
-      <c r="C2" s="0">
-        <v>0.20000000000000001</v>
-      </c>
-      <c r="D2" s="0">
-        <v>1</v>
-      </c>
-      <c r="E2" s="0">
+      <c r="C2">
+        <v>0.2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
         <v>0.01</v>
       </c>
-      <c r="F2" s="0">
+      <c r="F2">
         <v>100</v>
       </c>
-      <c r="G2" s="0">
+      <c r="G2">
         <v>10</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
-      <c r="A3" s="0" t="s">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="1">
         <v>46211.73766490478</v>
       </c>
-      <c r="C3" s="0">
-        <v>0.45000000000000001</v>
-      </c>
-      <c r="D3" s="0">
+      <c r="C3">
+        <v>0.45</v>
+      </c>
+      <c r="D3">
         <v>1.3</v>
       </c>
-      <c r="E3" s="0">
+      <c r="E3">
         <v>0.01</v>
       </c>
-      <c r="F3" s="0">
+      <c r="F3">
         <v>100</v>
       </c>
-      <c r="G3" s="0">
+      <c r="G3">
         <v>11.401754250991379</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
-      <c r="A4" s="0" t="s">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="1">
         <v>46211.739891338053</v>
       </c>
-      <c r="C4" s="0">
-        <v>0.45000000000000001</v>
-      </c>
-      <c r="D4" s="0">
+      <c r="C4">
+        <v>0.45</v>
+      </c>
+      <c r="D4">
         <v>1.3</v>
       </c>
-      <c r="E4" s="0">
+      <c r="E4">
         <v>0.01</v>
       </c>
-      <c r="F4" s="0">
+      <c r="F4">
         <v>100</v>
       </c>
-      <c r="G4" s="0">
+      <c r="G4">
         <v>11.401754250991379</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="1">
         <v>46212.822921438194</v>
       </c>
-      <c r="C5" s="0">
-        <v>0.20000000000000001</v>
-      </c>
-      <c r="D5" s="0">
-        <v>1</v>
-      </c>
-      <c r="E5" s="0">
+      <c r="C5">
+        <v>0.2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
         <v>0.01</v>
       </c>
-      <c r="F5" s="0">
+      <c r="F5">
         <v>100</v>
       </c>
-      <c r="G5" s="0">
+      <c r="G5">
+        <v>10</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46215.88352031714</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>0.01</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46215.883758330019</v>
+      </c>
+      <c r="C7">
+        <v>0.05</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0.01</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="G7">
         <v>10</v>
       </c>
     </row>
@@ -824,21 +937,187 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" customWidth="1"/>
+    <col min="4" max="4" width="8.77734375" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="4.77734375" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" customWidth="1"/>
+    <col min="11" max="11" width="4.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46212.802283827288</v>
+      </c>
+      <c r="C2">
+        <v>9.81</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>29.43</v>
+      </c>
+      <c r="I2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J2">
+        <v>1E-4</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46212.802345490047</v>
+      </c>
+      <c r="C3">
+        <v>9.81</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>29.43</v>
+      </c>
+      <c r="I3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J3">
+        <v>1E-4</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46212.802401839173</v>
+      </c>
+      <c r="C4">
+        <v>9.81</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>0.5</v>
+      </c>
+      <c r="H4">
+        <v>29.43</v>
+      </c>
+      <c r="I4">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J4">
+        <v>1E-4</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="true"/>
-    <col min="2" max="2" width="15.5546875" customWidth="true"/>
-    <col min="3" max="3" width="4.5546875" customWidth="true"/>
-    <col min="4" max="4" width="8.77734375" customWidth="true"/>
-    <col min="5" max="5" width="12.77734375" customWidth="true"/>
-    <col min="6" max="6" width="8" customWidth="true"/>
-    <col min="7" max="7" width="4.77734375" customWidth="true"/>
-    <col min="8" max="8" width="16.44140625" customWidth="true"/>
-    <col min="9" max="9" width="8.88671875" customWidth="true"/>
-    <col min="10" max="10" width="6.5546875" customWidth="true"/>
-    <col min="11" max="11" width="4.5546875" customWidth="true"/>
+    <col min="1" max="1" width="5.88671875" customWidth="true"/>
+    <col min="2" max="2" width="8.88671875" customWidth="true"/>
+    <col min="3" max="3" width="4.77734375" customWidth="true"/>
+    <col min="4" max="4" width="2.33203125" customWidth="true"/>
+    <col min="5" max="5" width="9.77734375" customWidth="true"/>
+    <col min="6" max="6" width="9.21875" customWidth="true"/>
+    <col min="7" max="7" width="10.6640625" customWidth="true"/>
+    <col min="8" max="8" width="12.33203125" customWidth="true"/>
+    <col min="9" max="9" width="12.33203125" customWidth="true"/>
+    <col min="10" max="10" width="11.77734375" customWidth="true"/>
+    <col min="11" max="11" width="11.77734375" customWidth="true"/>
+    <col min="12" max="12" width="2" customWidth="true"/>
+    <col min="13" max="13" width="4.6640625" customWidth="true"/>
+    <col min="14" max="14" width="16.109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -849,136 +1128,84 @@
         <v>2</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="J1" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="0" t="s">
-        <v>21</v>
+      <c r="M1" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1">
-        <v>46212.802283827288</v>
+        <v>46217.72499059861</v>
       </c>
       <c r="C2" s="0">
-        <v>9.8100000000000005</v>
+        <v>2</v>
       </c>
       <c r="D2" s="0">
         <v>3</v>
       </c>
       <c r="E2" s="0">
-        <v>1</v>
+        <v>1200</v>
       </c>
       <c r="F2" s="0">
-        <v>10</v>
+        <v>800</v>
       </c>
       <c r="G2" s="0">
-        <v>1</v>
+        <v>0.17453292519943295</v>
       </c>
       <c r="H2" s="0">
-        <v>29.43</v>
+        <v>2000</v>
       </c>
       <c r="I2" s="0">
-        <v>1.0000000000000001e-05</v>
+        <v>100</v>
       </c>
       <c r="J2" s="0">
-        <v>0.0001</v>
+        <v>-7000</v>
       </c>
       <c r="K2" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="1">
-        <v>46212.802345490047</v>
-      </c>
-      <c r="C3" s="0">
-        <v>9.8100000000000005</v>
-      </c>
-      <c r="D3" s="0">
-        <v>3</v>
-      </c>
-      <c r="E3" s="0">
-        <v>1</v>
-      </c>
-      <c r="F3" s="0">
-        <v>10</v>
-      </c>
-      <c r="G3" s="0">
-        <v>2</v>
-      </c>
-      <c r="H3" s="0">
-        <v>29.43</v>
-      </c>
-      <c r="I3" s="0">
-        <v>1.0000000000000001e-05</v>
-      </c>
-      <c r="J3" s="0">
-        <v>0.0001</v>
-      </c>
-      <c r="K3" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="1">
-        <v>46212.802401839173</v>
-      </c>
-      <c r="C4" s="0">
-        <v>9.8100000000000005</v>
-      </c>
-      <c r="D4" s="0">
-        <v>3</v>
-      </c>
-      <c r="E4" s="0">
-        <v>1</v>
-      </c>
-      <c r="F4" s="0">
-        <v>10</v>
-      </c>
-      <c r="G4" s="0">
-        <v>0.5</v>
-      </c>
-      <c r="H4" s="0">
-        <v>29.43</v>
-      </c>
-      <c r="I4" s="0">
-        <v>1.0000000000000001e-05</v>
-      </c>
-      <c r="J4" s="0">
-        <v>0.0001</v>
-      </c>
-      <c r="K4" s="0">
-        <v>0</v>
+        <v>-10000</v>
+      </c>
+      <c r="L2" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="M2" s="0">
+        <v>-0.4537856055185257</v>
+      </c>
+      <c r="N2" s="0">
+        <v>294.30000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>